<commit_message>
update logic on Simple_calculation. fix on feeders logic, update extra line item in mainrule table for exceed range qty
</commit_message>
<xml_diff>
--- a/config/MainConfig.xlsx
+++ b/config/MainConfig.xlsx
@@ -12882,7 +12882,9 @@
     <col min="1" max="1" width="33.1428571428571" style="1" customWidth="1"/>
     <col min="2" max="2" width="96.1428571428571" style="1" customWidth="1"/>
     <col min="3" max="3" width="33.1428571428571" style="1" customWidth="1"/>
-    <col min="4" max="6" width="10.2857142857143" style="1"/>
+    <col min="4" max="4" width="23.1428571428571" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.4285714285714" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.2857142857143" style="1"/>
     <col min="7" max="7" width="13.5714285714286" style="1" customWidth="1"/>
     <col min="8" max="9" width="10.2857142857143" style="1"/>
     <col min="10" max="10" width="62.5714285714286" style="1" customWidth="1"/>

</xml_diff>